<commit_message>
audit log week 4 and week 5
</commit_message>
<xml_diff>
--- a/AI Audit Log_HoThiLinhGiang.xlsx
+++ b/AI Audit Log_HoThiLinhGiang.xlsx
@@ -1,43 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\KÌ 7\SWD392\nopbaitap\ai-audit-log-tuilavetne\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05795F0A-6AA6-4423-9062-3B79C89F384C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4542B6E9-4BF0-45FF-9D47-B4FCCE8D85A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{84C35D15-8A6C-4EDA-8B49-2CCD89DED56E}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="3" xr2:uid="{84C35D15-8A6C-4EDA-8B49-2CCD89DED56E}"/>
   </bookViews>
   <sheets>
     <sheet name="Week 2" sheetId="1" r:id="rId1"/>
     <sheet name="Week 3" sheetId="2" r:id="rId2"/>
-    <sheet name="Assignment 2" sheetId="3" r:id="rId3"/>
-    <sheet name="Assignment 3" sheetId="4" r:id="rId4"/>
+    <sheet name="Week 4" sheetId="3" r:id="rId3"/>
+    <sheet name="Week 5" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="58">
   <si>
     <t>Giai đoạn/Thành phần DTC</t>
   </si>
@@ -669,19 +660,143 @@
       </rPr>
       <t xml:space="preserve"> Khớp hoàn toàn với yêu cầu "inherit from it" của đề bài.</t>
     </r>
+  </si>
+  <si>
+    <t>Slot 9</t>
+  </si>
+  <si>
+    <t>Slot 7</t>
+  </si>
+  <si>
+    <t>"Làm thế nào để thể hiện các DTO (Data
+Transfer Object) trong Class Diagram cho User Management Feature?"</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI giải thích DTO nên được tách thành các lớp riêng biệt 
+(như CreateUserDTO, UpdateUserDTO) và thể hiện bằng mũi tên Dependency từ Controller/Service đến DTO.
+Quyết định: Tôi thêm các DTO vào diagram để làm rõ luồng dữ liệu truyền giữa client và backend, tránh việc dùng trực tiếp Entity cho Request/Response.</t>
+  </si>
+  <si>
+    <t>"Phân tích quan hệ giữa Order và OrderItem: nên dùng Composition (hình thoi đặc) hay Aggregation (hình thoi rỗng)?"</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI phân tích rằng OrderItem không thể tồn tại độc lập nếu
+thiếu Order, do đó quan hệ Composition là chính xác nhất về mặt nghiệp vụ.
+Quyết định: Tôi điều chỉnh lại nét vẽ trên UML thành Composition để phản ánh đúng logic xóa cascade (xóa Order thì xóa luôn OrderItem).</t>
+  </si>
+  <si>
+    <t>"Cách biểu diễn kiểu dữ liệu Enum (ví dụ:
+UserRole gồm ADMIN, USER) chuẩn xác nhất trong Class Diagram là gì?"</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI hướng dẫn sử dụng stereotype &lt;&lt;enumeration&gt;&gt; cho 1
+block riêng và dùng nét đứt (dependency) hoặc association để nối vào User Entity.
+Quyết định: Tôi tạo một block Enum riêng trên PlantUML để làm rõ các phân quyền thay vì chỉ để kiểu String trong thuộc tính role.</t>
+  </si>
+  <si>
+    <t>"Khi nào nên dùng Interface và khi nào
+dùng Abstract Class trong thiết kế Service layer? Sinh ví dụ bằng PlantUML."</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI phân biệt: Interface dùng để định nghĩa contract (hành vi), Abstract Class dùng khi có logic dùng chung. AI cung cấp code PlantUML minh họa.
+Quyết định: Tôi áp dụng Interface cho IUserService để tuân thủ Dependency Inversion và giúp việc mock data khi viết Unit Test dễ dàng hơn.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Đánh giá mức độ coupling giữa UserController và EmailService trong biểu đồ hiện tại. Đề xuất cách giảm coupling."
+</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI chỉ ra việc Controller gọi trực tiếp service bên ngoài làm tăng coupling, đề xuất sử dụng Interface hoặc cơ chế Event-Driven.
+Quyết định: Tôi cập nhật Class Diagram, bổ sung IEmailService để decouple, giúp kiến trúc linh hoạt hơn nếu sau này đổi provider gửi mail.</t>
+  </si>
+  <si>
+    <t>"Kiểm tra cách thể hiện quan hệ One-to-
+many và Many-to-Many giữa User và Role trong Class Diagram (áp dụng với TypeORM)."</t>
+  </si>
+  <si>
+    <t>Phản hồi: Ai giải thích cách đặt multiplicity (1 to 0..* hoặc * to *) và
+gợi ý việc có nên hiển thị bảng trung gian (JoinTable) trên biểu đồ hay không.
+Quyết định: Với mức logic nghiệp vụ, tôi ẩn bảng trung gian và dùng multiplicity *..*. Nhưng tôi ghi chú lại để xử lý khi cấu hình Entity trong code.</t>
+  </si>
+  <si>
+    <t>"Phân biệt Repository pattern và DAO 
+pattern trong Class Diagram. Kiến trúc hiện tại của dự án nên dùng cái nào?"</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI giải thích DAO thường map trực tiếp 1-1 với DB table, 
+trong khi Repository làm việc với Domain Entity (chứa logic nghiệp vụ).
+Quyết định: Tôi quyết định sử dụng tên gọi và cấu trúc của Repository để đồng nhất với các framework/ORM hiện đại đang sử dụng.</t>
+  </si>
+  <si>
+    <t>"Các lớp Custom Exception (như NotFoundException,UnauthorizedException) có cần thiết phải vẽ vào Class Diagram không?"</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI khuyên chỉ nên đưa vào nếu Exception đó mang logic
+nghiệp vụ cốt lõi, còn lại không nên vẽ để tránh làm biểu đồ bị rối (cluttered).
+Quyết định: Tôi lược bỏ các Exception cơ bản khỏi Class Diagram tổng thể để giữ biểu đồ clean, tập trung vào Entity và Service chính.</t>
+  </si>
+  <si>
+    <t>"Phân tích luồng gọi API từ Client (Frontend
+React) đến Backend ExpressJS (qua các lớp Controller -&gt; Service -&gt; Repository) cho chức năng Đăng ký tài khoản."</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI mô tả thứ tự gọi hàm tuần tự giữa các lifeline
+(đường đời) nhấn mạnh việc Controller nhận request, Service xử lý nghiệp vụ và Repository thao tác với DB.
+Quyết định: Tôi dùng luồng này làm template chuẩn cho mọi API CRUD cơ bản trong báo cáo đồ án.</t>
+  </si>
+  <si>
+    <t>"Làm sao để thể hiện middleware (ví dụ: verifyToken dùng để check JWT) trong Sequence Diagram trước khi request thực sự đi vào Controller?"</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI gợi ý đặt middleware như 1 lifeline trung gian giữa
+Route/Router và Controller, sử dụng khối opt hoặc trả về lỗi 401 ngay lập tức nếu token không hợp lệ.
+Quyết định: Tôi bổ sung lifeline AuthMiddleware để làm rõ luồng bảo mật, sát với source code thực tế.</t>
+  </si>
+  <si>
+    <t>"Vẽ Sequence Diagram cho chức năng đăng
+nhập. Hướng dẫn cách sử dụng alt fragment để xử lý hai trường hợp phân nhánh: Sai mật khẩu và Đăng nhập thành công."</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI giải thích cú pháp khung alt/else trong UML để bọc
+các luồng xử lý điều kiện if/else.
+Quyết định: Tôi áp dụng alt để tách bạch rõ ràng thông điệp trả về (Error message vs. Trả về Access Token).</t>
+  </si>
+  <si>
+    <t>"Thể hiện việc hệ thống gọi ra 1 external system (ví dụ: Gọi API của VNPay để thanh toán hoặc Nodemailer để gửi email OTP) trong Sequence Diagram như thế nào?"</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI khuyên nên tạo 1 actor/lifeline nằm ngoài cùng
+bên phải với stereotype &lt;&lt;External System&gt;&gt; và dùng nét đứt để biểu diễn kết quả trả về chậm (callback).
+Quyết định: Tôi phân định rõ ranh giới hệ thống, giúp thấy rõ service nào đang phụ thuộc vào bên thứ ba.</t>
+  </si>
+  <si>
+    <t>"Sinh mã PlantUML cho sequence diagram
+chức năng Reset Password (Quên mật khẩu), bao gồm các lifeline: User, Client, AuthController, UserService, EmailService."</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI cung cấp code PlantUML với cấu trúc khai báo
+actor, boundary, control, entity và các mũi tên -&gt;, --&gt;.
+Quyết định: Tôi tái sử dụng và tinh chỉnh mã này để chèn thẳng vào tài liệu phân tích thiết kế, tiết kiệm thời gian vẽ tay.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <charset val="163"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -753,7 +868,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -762,23 +877,23 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Bình thường" xfId="0" builtinId="0"/>
@@ -1238,100 +1353,100 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="9" t="s">
+      <c r="B1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="9" t="s">
+      <c r="C1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="9" t="s">
+      <c r="D1" s="4" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="72" x14ac:dyDescent="0.3">
-      <c r="A2" s="10">
+      <c r="A2" s="9">
         <v>1</v>
       </c>
-      <c r="B2" s="10" t="s">
+      <c r="B2" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="C2" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="D2" s="13" t="s">
+      <c r="D2" s="11" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="72" x14ac:dyDescent="0.3">
-      <c r="A3" s="10">
+      <c r="A3" s="9">
         <v>2</v>
       </c>
-      <c r="B3" s="10" t="s">
+      <c r="B3" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="12" t="s">
+      <c r="C3" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="D3" s="13" t="s">
+      <c r="D3" s="11" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A4" s="10">
+      <c r="A4" s="9">
         <v>3</v>
       </c>
-      <c r="B4" s="10" t="s">
+      <c r="B4" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="C4" s="12" t="s">
+      <c r="C4" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="D4" s="13" t="s">
+      <c r="D4" s="11" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="A5" s="10">
+      <c r="A5" s="9">
         <v>4</v>
       </c>
-      <c r="B5" s="10" t="s">
+      <c r="B5" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="C5" s="12" t="s">
+      <c r="C5" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="D5" s="13" t="s">
+      <c r="D5" s="11" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="115.2" x14ac:dyDescent="0.3">
-      <c r="A6" s="10">
+      <c r="A6" s="9">
         <v>5</v>
       </c>
-      <c r="B6" s="10" t="s">
+      <c r="B6" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="C6" s="12" t="s">
+      <c r="C6" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="D6" s="13" t="s">
+      <c r="D6" s="11" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="129.6" x14ac:dyDescent="0.3">
-      <c r="A7" s="11">
+      <c r="A7" s="9">
         <v>6</v>
       </c>
-      <c r="B7" s="10" t="s">
+      <c r="B7" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="C7" s="12" t="s">
+      <c r="C7" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="D7" s="13" t="s">
+      <c r="D7" s="11" t="s">
         <v>27</v>
       </c>
     </row>
@@ -1342,18 +1457,282 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{69A16565-6ACB-4DDB-B0C1-55C7722368A3}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
+  <cols>
+    <col min="2" max="2" width="27.6640625" customWidth="1"/>
+    <col min="3" max="3" width="33" customWidth="1"/>
+    <col min="4" max="4" width="54.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A2" s="9">
+        <v>1</v>
+      </c>
+      <c r="B2" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C2" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="D2" s="12" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A3" s="9">
+        <v>2</v>
+      </c>
+      <c r="B3" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="D3" s="10" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A4" s="9">
+        <v>3</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="D4" s="10" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A5" s="9">
+        <v>4</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C5" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="D5" s="10" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A6" s="9">
+        <v>5</v>
+      </c>
+      <c r="B6" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C6" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="D6" s="10" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A7" s="9">
+        <v>6</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C7" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="D7" s="10" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A8" s="9">
+        <v>7</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C8" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="D8" s="10" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="72" x14ac:dyDescent="0.3">
+      <c r="A9" s="9">
+        <v>8</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C9" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="D9" s="10" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A10" s="13"/>
+      <c r="B10" s="13"/>
+      <c r="C10" s="13"/>
+      <c r="D10" s="13"/>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A11" s="13"/>
+      <c r="B11" s="13"/>
+      <c r="C11" s="13"/>
+      <c r="D11" s="13"/>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{323516A4-AE23-41CF-AD84-97A6064FC5FB}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
+  <cols>
+    <col min="2" max="2" width="26.33203125" customWidth="1"/>
+    <col min="3" max="3" width="36.6640625" customWidth="1"/>
+    <col min="4" max="4" width="50.109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="72" x14ac:dyDescent="0.3">
+      <c r="A2" s="9">
+        <v>1</v>
+      </c>
+      <c r="B2" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="C2" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="D2" s="10" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A3" s="9">
+        <v>2</v>
+      </c>
+      <c r="B3" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="D3" s="10" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="72" x14ac:dyDescent="0.3">
+      <c r="A4" s="9">
+        <v>3</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="D4" s="10" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="72" x14ac:dyDescent="0.3">
+      <c r="A5" s="9">
+        <v>4</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="C5" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="D5" s="10" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A6" s="9">
+        <v>5</v>
+      </c>
+      <c r="B6" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="C6" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="D6" s="10" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" s="13"/>
+      <c r="B7" s="13"/>
+      <c r="C7" s="13"/>
+      <c r="D7" s="13"/>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" s="13"/>
+      <c r="B8" s="13"/>
+      <c r="C8" s="13"/>
+      <c r="D8" s="13"/>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9" s="13"/>
+      <c r="B9" s="13"/>
+      <c r="C9" s="13"/>
+      <c r="D9" s="13"/>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A10" s="13"/>
+      <c r="B10" s="13"/>
+      <c r="C10" s="13"/>
+      <c r="D10" s="13"/>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A11" s="13"/>
+      <c r="B11" s="13"/>
+      <c r="C11" s="13"/>
+      <c r="D11" s="13"/>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
audit log week 6
</commit_message>
<xml_diff>
--- a/AI Audit Log_HoThiLinhGiang.xlsx
+++ b/AI Audit Log_HoThiLinhGiang.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\KÌ 7\SWD392\nopbaitap\ai-audit-log-tuilavetne\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4542B6E9-4BF0-45FF-9D47-B4FCCE8D85A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E63D4F91-C75C-42E6-A7EB-23A81023F0BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="3" xr2:uid="{84C35D15-8A6C-4EDA-8B49-2CCD89DED56E}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11628" windowHeight="12336" firstSheet="1" activeTab="4" xr2:uid="{84C35D15-8A6C-4EDA-8B49-2CCD89DED56E}"/>
   </bookViews>
   <sheets>
     <sheet name="Week 2" sheetId="1" r:id="rId1"/>
     <sheet name="Week 3" sheetId="2" r:id="rId2"/>
     <sheet name="Week 4" sheetId="3" r:id="rId3"/>
     <sheet name="Week 5" sheetId="4" r:id="rId4"/>
+    <sheet name="Week 6" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -28,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="79">
   <si>
     <t>Giai đoạn/Thành phần DTC</t>
   </si>
@@ -777,19 +778,113 @@
     <t>Phản hồi: AI cung cấp code PlantUML với cấu trúc khai báo
 actor, boundary, control, entity và các mũi tên -&gt;, --&gt;.
 Quyết định: Tôi tái sử dụng và tinh chỉnh mã này để chèn thẳng vào tài liệu phân tích thiết kế, tiết kiệm thời gian vẽ tay.</t>
+  </si>
+  <si>
+    <t>Slot 11</t>
+  </si>
+  <si>
+    <t>"Hãy giải thích State Diagram trong UML. 
+Nó được dùng để mô hình hóa điều gì trong hệ thống phần mềm?"</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI giải thích state diagram là 1 loại behavioral diagram trong UML, dùng để mô tả các trạng thái của một object và sự chuyển đổi giữa các trạng thái đó theo thời gian, dựa trên event. Nó đặc biệt phù hợp với các object có vòng đời rõ ràng như Order, User Session hoặc Payment.
+Quyết định: Tôi sử dụng state diagram để mô hình hóa các object có hành vi thay đổi theo trạng thái trong hệ thống, giúp hiểu rõ lifecycle thay vì chỉ nhìn vào class structure.</t>
+  </si>
+  <si>
+    <t>"Trong state diagram, state là gì? Hãy hướng dẫn cách xác định state cho 1 object"</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI cho rằng state là 1 condition mà object tồn tại trong 1 khoảng thời gian và có thể phản ứng với event. State thường được xác định từ business status hoặc các giai đoạn xử lý.
+Quyết định: Tôi xác định state dựa trên nghiệp vụ thực tế như Pending, Processing, Completed thay vì chỉ dựa vào attribute đơn lẻ.</t>
+  </si>
+  <si>
+    <t>"Event trong state diagram là gì? Nó ảnh
+hưởng đến transition như thế nào?"</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI giải thích event là 1 sự kiện xảy ra tại 1 thời điểm
+và có thể kích hoạt transition giữa các state. Transition thể hiện sự thay đổi trạng thái do event gây ra.
+Quyết định: Tôi luôn ghi rõ event trên các transition như submitOrder, cancelOrder, confirmPayment để đảm bảo sơ đồ rõ ràng và đúng logic hệ thống.</t>
+  </si>
+  <si>
+    <t>"Guard condition trong state diagram là gì? Khi nào nên sử dụng?"</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI giải thích guard condition là điều kiện boolean đi
+kèm event, chỉ khi điều kiện đúng thì transition mới xảy ra. Ví dụ: confirmPayment [amount &gt;= total].
+Quyết định: Tôi sử dụng guard condition để tránh sai logic nghiệp vụ, đặc biệt trong các trường hợp kiểm tra dữ liệu trước khi chuyển state.</t>
+  </si>
+  <si>
+    <t>"Phân biệt entry action và exit action trong
+state diagram"</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI cho biết entry action được thực hiện khi vào state, 
+exit action khi rời state. Điều này giúp tránh lặp lại action ở nhiều transition.
+Quyết định: Tôi áp dụng entry action cho các xử lý chung như entry/Completed: sendNotification() để tối ưu sơ đồ.</t>
+  </si>
+  <si>
+    <t>"Hãy giải thích Activity Diagram trong UML 
+và mục đích sử dụng"</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI mô tả activity diagram dùng để biểu diễn workflow
+hoặc luồng xử lý của hệ thống, từ bước bắt đầu đến kết thúc, bao gồm các nhánh điều kiện và song song.
+Quyết định: Tôi dùng activity diagram để mô tả business process thay vì hành vi từng object như state diagram.</t>
+  </si>
+  <si>
+    <t>"Decision node và merge node trong activity diagram có vai trò gì?"</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI giải thích decision node dùng để rẽ nhánh theo
+điều kiện, còn merge node dùng để hợp các nhánh lại.
+Quyết định: Tôi sử dụng decision node cho các trường hợp if/else và merge node để đảm bảo luồng không bị rối hoặc sai logic.</t>
+  </si>
+  <si>
+    <t>"Fork và join trong activity diagram dùng
+để làm gì?"</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI cho biết fork dùng để tách luồng thành các hoạt
+động song song, join dùng để đồng bộ lại các luồng đó.
+Quyết định: Tôi áp dụng fork/join khi hệ thống thực hiện nhiều tác vụ cùng lúc như gửi email và lưu dữ liệu.</t>
+  </si>
+  <si>
+    <t>"Swimlane trong activity diagram có ý 
+nghĩa gì?"</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI giải thích swimlane dùng để phân chia trách nhiệm
+giữa các actor hoặc hệ thống con.
+Quyết định: Tôi sử dụng swimlane để thể hiện rõ ai thực hiện bước nào (User, System, Admin), giúp dễ hiểu hơn khi trình bày.</t>
+  </si>
+  <si>
+    <t>"So sánh State Diagram và Activity Diagram, khi nào nên dùng mỗi loại?"</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI chỉ ra state diagram tập trung vào trạng thái của 
+object, còn activity diagram tập trung vào luồng xử lý. State diagram phù hợp với lifecycle, activity diagram phù hợp với workflow.
+Quyết định: Tôi kết hợp cả hai loại biểu đồ: dùng state diagram cho object quan trọng (Order, Payment) và activity diagram cho các quy trình nghiệp vụ (Place Order, Payment Process).</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <charset val="163"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -857,7 +952,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -868,7 +963,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -877,23 +972,22 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Bình thường" xfId="0" builtinId="0"/>
@@ -1457,7 +1551,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{69A16565-6ACB-4DDB-B0C1-55C7722368A3}">
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="27.6640625" customWidth="1"/>
@@ -1591,18 +1685,6 @@
         <v>47</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A10" s="13"/>
-      <c r="B10" s="13"/>
-      <c r="C10" s="13"/>
-      <c r="D10" s="13"/>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A11" s="13"/>
-      <c r="B11" s="13"/>
-      <c r="C11" s="13"/>
-      <c r="D11" s="13"/>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1610,7 +1692,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{323516A4-AE23-41CF-AD84-97A6064FC5FB}">
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="26.33203125" customWidth="1"/>
@@ -1702,35 +1784,174 @@
         <v>57</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A7" s="13"/>
-      <c r="B7" s="13"/>
-      <c r="C7" s="13"/>
-      <c r="D7" s="13"/>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A8" s="13"/>
-      <c r="B8" s="13"/>
-      <c r="C8" s="13"/>
-      <c r="D8" s="13"/>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A9" s="13"/>
-      <c r="B9" s="13"/>
-      <c r="C9" s="13"/>
-      <c r="D9" s="13"/>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A10" s="13"/>
-      <c r="B10" s="13"/>
-      <c r="C10" s="13"/>
-      <c r="D10" s="13"/>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A11" s="13"/>
-      <c r="B11" s="13"/>
-      <c r="C11" s="13"/>
-      <c r="D11" s="13"/>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EFAE320A-C878-4365-9536-22BE82E94BCF}">
+  <dimension ref="A1:D11"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="31.21875" customWidth="1"/>
+    <col min="3" max="3" width="34" customWidth="1"/>
+    <col min="4" max="4" width="50.109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="115.2" x14ac:dyDescent="0.3">
+      <c r="A2" s="9">
+        <v>1</v>
+      </c>
+      <c r="B2" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C2" s="10" t="s">
+        <v>59</v>
+      </c>
+      <c r="D2" s="10" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A3" s="9">
+        <v>2</v>
+      </c>
+      <c r="B3" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>61</v>
+      </c>
+      <c r="D3" s="10" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A4" s="9">
+        <v>3</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="D4" s="10" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A5" s="9">
+        <v>4</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C5" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="D5" s="10" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A6" s="9">
+        <v>5</v>
+      </c>
+      <c r="B6" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C6" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="D6" s="10" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A7" s="9">
+        <v>6</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C7" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="D7" s="10" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="72" x14ac:dyDescent="0.3">
+      <c r="A8" s="9">
+        <v>7</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C8" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="D8" s="10" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A9" s="9">
+        <v>8</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C9" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="D9" s="10" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A10" s="9">
+        <v>9</v>
+      </c>
+      <c r="B10" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C10" s="10" t="s">
+        <v>75</v>
+      </c>
+      <c r="D10" s="10" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="115.2" x14ac:dyDescent="0.3">
+      <c r="A11" s="9">
+        <v>10</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C11" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="D11" s="10" t="s">
+        <v>78</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>